<commit_message>
Progress on template file creation for n loops out_last_timestep
</commit_message>
<xml_diff>
--- a/CryoGrid/CryoGridCommunity_results/templates/save_last_timestep_nloop/save_last_timestep_nloop.xlsx
+++ b/CryoGrid/CryoGridCommunity_results/templates/save_last_timestep_nloop/save_last_timestep_nloop.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\templates\save_last_timestep_nloop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D927A1CC-BD0C-4FBE-928B-9FAB52E70D43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72043211-4050-4FB1-8C8F-6776A78F4CA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4188" yWindow="-17388" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="216">
   <si>
     <t>-------------------</t>
   </si>
@@ -540,9 +540,6 @@
     <t>skyview_factor</t>
   </si>
   <si>
-    <t>TILE_1D_standard2</t>
-  </si>
-  <si>
     <t>init_steady_state_class</t>
   </si>
   <si>
@@ -570,12 +567,6 @@
     <t>Trying -2C everywhere</t>
   </si>
   <si>
-    <t>you need an additional first tile, which has "new_init" as builder, followed by 9x the same run, but with "update_forcing_out" as builder.</t>
-  </si>
-  <si>
-    <t>in your configuration, you would restart the same simulation from the initial T-profile 10x, so the first 9 runs would essentially do nothing, and you end up with only 10 years of spinup!</t>
-  </si>
-  <si>
     <t>I would always assume saturated conditions in the layers that are expected to be permafrost, like water+mineral = 1</t>
   </si>
   <si>
@@ -688,6 +679,9 @@
   </si>
   <si>
     <t>D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\forcing\Forcing_Data\</t>
+  </si>
+  <si>
+    <t>TILE_1D</t>
   </si>
 </sst>
 </file>
@@ -1161,7 +1155,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -1191,20 +1185,18 @@
         <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="D6" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="E6" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="F6" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="10" t="s">
-        <v>178</v>
-      </c>
+      <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -1225,13 +1217,11 @@
       <c r="F7" t="s">
         <v>24</v>
       </c>
-      <c r="G7" s="10" t="s">
-        <v>179</v>
-      </c>
+      <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B8" t="s">
         <v>21</v>
@@ -1334,7 +1324,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="4"/>
@@ -1366,7 +1356,7 @@
     </row>
     <row r="28" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A28" s="9" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="B28" s="9">
         <v>1</v>
@@ -1378,7 +1368,7 @@
         <v>8</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="31" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1389,7 +1379,7 @@
         <v>100</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="32" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1432,7 +1422,7 @@
         <v>21</v>
       </c>
       <c r="C36" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D36" t="s">
         <v>24</v>
@@ -1485,7 +1475,7 @@
         <v>24</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="41" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1513,7 +1503,7 @@
         <v>27</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="43" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1538,7 +1528,7 @@
         <v>24</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="45" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1557,37 +1547,37 @@
     </row>
     <row r="46" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="47" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="48" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B48">
         <v>-2</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="49" spans="1:5" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B49">
         <v>0.5</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="50" spans="1:5" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1614,7 +1604,7 @@
     </row>
     <row r="55" spans="1:5" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A55" s="9" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="B55" s="9">
         <v>2</v>
@@ -1626,15 +1616,15 @@
         <v>8</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="58" spans="1:5" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C58" s="9"/>
       <c r="D58" s="9"/>
@@ -1642,10 +1632,10 @@
     </row>
     <row r="59" spans="1:5" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C59" s="9"/>
       <c r="D59" s="9"/>
@@ -1659,7 +1649,7 @@
         <v>21</v>
       </c>
       <c r="C60" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="D60" t="s">
         <v>24</v>
@@ -1683,7 +1673,7 @@
     </row>
     <row r="62" spans="1:5" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C62" s="9"/>
       <c r="D62" s="9"/>
@@ -1691,7 +1681,7 @@
     </row>
     <row r="63" spans="1:5" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C63" s="5"/>
       <c r="D63" s="5"/>
@@ -1724,7 +1714,7 @@
     </row>
     <row r="70" spans="1:5" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A70" s="9" t="s">
-        <v>168</v>
+        <v>215</v>
       </c>
       <c r="B70" s="9">
         <v>3</v>
@@ -1736,7 +1726,7 @@
         <v>8</v>
       </c>
       <c r="B72" s="9" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
     </row>
     <row r="73" spans="1:5" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1763,7 +1753,7 @@
         <v>21</v>
       </c>
       <c r="C75" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D75" t="s">
         <v>24</v>
@@ -1828,7 +1818,7 @@
         <v>32</v>
       </c>
       <c r="B83" s="16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C83" s="14"/>
       <c r="D83" s="14"/>
@@ -1840,7 +1830,7 @@
         <v>33</v>
       </c>
       <c r="B84" s="17" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C84" s="14"/>
       <c r="D84" s="14"/>
@@ -2008,7 +1998,7 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B103">
         <v>1</v>
@@ -2021,7 +2011,7 @@
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B105">
         <v>5</v>
@@ -2030,7 +2020,7 @@
         <v>5</v>
       </c>
       <c r="D105" s="8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.35">
@@ -2053,7 +2043,7 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B111">
         <v>1</v>
@@ -2061,13 +2051,13 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B113">
         <v>5</v>
       </c>
       <c r="D113" s="8" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.35">
@@ -2075,7 +2065,7 @@
         <v>43</v>
       </c>
       <c r="B114" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D114" s="8"/>
     </row>
@@ -2099,7 +2089,7 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B120">
         <v>2</v>
@@ -2107,13 +2097,13 @@
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B122">
         <v>5</v>
       </c>
       <c r="D122" s="8" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.35">
@@ -2121,7 +2111,7 @@
         <v>43</v>
       </c>
       <c r="B123" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D123" s="8"/>
     </row>
@@ -2370,7 +2360,7 @@
         <v>2</v>
       </c>
       <c r="D157" s="10" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="158" spans="1:10" x14ac:dyDescent="0.35">
@@ -2381,7 +2371,7 @@
         <v>1</v>
       </c>
       <c r="D158" s="10" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="160" spans="1:10" x14ac:dyDescent="0.35">
@@ -2490,7 +2480,7 @@
         <v>24</v>
       </c>
       <c r="G164" s="10" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.35">
@@ -2498,12 +2488,12 @@
         <v>6</v>
       </c>
       <c r="G165" s="10" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="166" spans="1:8" x14ac:dyDescent="0.35">
       <c r="G166" s="10" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="167" spans="1:8" s="14" customFormat="1" x14ac:dyDescent="0.35"/>
@@ -2569,7 +2559,7 @@
         <v>-2</v>
       </c>
       <c r="D174" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="175" spans="1:8" x14ac:dyDescent="0.35">
@@ -2681,7 +2671,7 @@
         <v>0.1</v>
       </c>
       <c r="D186" s="8" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.35">
@@ -2695,7 +2685,7 @@
         <v>0.1</v>
       </c>
       <c r="D187" s="8" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.35">
@@ -2709,7 +2699,7 @@
         <v>0.5</v>
       </c>
       <c r="D188" s="8" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.35">
@@ -2723,7 +2713,7 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="D189" s="8" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.35">
@@ -2936,7 +2926,7 @@
         <v>0</v>
       </c>
       <c r="D209" s="8" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.35">
@@ -3120,7 +3110,7 @@
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B228">
         <v>0</v>
@@ -3129,7 +3119,7 @@
         <v>0</v>
       </c>
       <c r="D228" s="8" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.35">
@@ -3195,7 +3185,7 @@
         <v>102</v>
       </c>
       <c r="C233" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D233" s="8" t="s">
         <v>78</v>

</xml_diff>